<commit_message>
chore(weekly-sync): auto-pull through 2026-07-20
</commit_message>
<xml_diff>
--- a/data/ams_weekly_data/Audio_Array/ads_report_week29.xlsx
+++ b/data/ams_weekly_data/Audio_Array/ads_report_week29.xlsx
@@ -986,10 +986,10 @@
         <v>70076</v>
       </c>
       <c r="G20" t="n">
-        <v>54097.43</v>
+        <v>57062.68</v>
       </c>
       <c r="H20" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="21">
@@ -1826,10 +1826,10 @@
         <v>178351</v>
       </c>
       <c r="G50" t="n">
-        <v>9568.620000000001</v>
+        <v>10627.09</v>
       </c>
       <c r="H50" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="51">
@@ -1938,10 +1938,10 @@
         <v>39050</v>
       </c>
       <c r="G54" t="n">
-        <v>11094.9</v>
+        <v>9485.58</v>
       </c>
       <c r="H54" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="55">
@@ -2162,10 +2162,10 @@
         <v>38179</v>
       </c>
       <c r="G62" t="n">
-        <v>38172.86</v>
+        <v>44527.94</v>
       </c>
       <c r="H62" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="63">
@@ -7594,10 +7594,10 @@
         <v>33864</v>
       </c>
       <c r="G256" t="n">
-        <v>10253.33</v>
+        <v>12667.74</v>
       </c>
       <c r="H256" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="257">
@@ -8462,10 +8462,10 @@
         <v>2408</v>
       </c>
       <c r="G287" t="n">
-        <v>0</v>
+        <v>8472.030000000001</v>
       </c>
       <c r="H287" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="288">
@@ -8689,7 +8689,7 @@
         <v>18555.94</v>
       </c>
       <c r="H295" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="296">
@@ -8770,10 +8770,10 @@
         <v>24140</v>
       </c>
       <c r="G298" t="n">
-        <v>12964.41</v>
+        <v>21096.61</v>
       </c>
       <c r="H298" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="299">
@@ -9078,10 +9078,10 @@
         <v>1872</v>
       </c>
       <c r="G309" t="n">
-        <v>5338.14</v>
+        <v>12116.95</v>
       </c>
       <c r="H309" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="310">
@@ -9162,10 +9162,10 @@
         <v>12941</v>
       </c>
       <c r="G312" t="n">
-        <v>3219.49</v>
+        <v>7285.59</v>
       </c>
       <c r="H312" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="313">
@@ -9498,10 +9498,10 @@
         <v>8410</v>
       </c>
       <c r="G324" t="n">
-        <v>4235.6</v>
+        <v>6099.16</v>
       </c>
       <c r="H324" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="325">
@@ -11155,7 +11155,7 @@
         <v>371.3349985674643</v>
       </c>
       <c r="G2" t="n">
-        <v>1265.412866299392</v>
+        <v>1289.211787395323</v>
       </c>
       <c r="H2" t="n">
         <v>1</v>
@@ -11188,10 +11188,10 @@
         <v>8210.325001432537</v>
       </c>
       <c r="G3" t="n">
-        <v>27978.64713370061</v>
+        <v>28504.84821260468</v>
       </c>
       <c r="H3" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>

</xml_diff>